<commit_message>
First pass updates for autumn 2026
</commit_message>
<xml_diff>
--- a/files/grading_scale.xlsx
+++ b/files/grading_scale.xlsx
@@ -1,21 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10312"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://buckeyemailosu-my.sharepoint.com/personal/cooperstone_1_osu_edu/Documents/BuckeyeBox Data/JLC_Files/OSU/teaching/data-viz/dataviz-site/files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jessicacooperstone/git/rdataviz/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70AE761E-A126-CB47-B079-89BECD4733CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD34BFB3-A266-1F46-BCD6-F74B52F6AD99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="15560" yWindow="2120" windowWidth="28040" windowHeight="16940" xr2:uid="{31371ACA-339D-F64C-9977-84D6DF8EF93B}"/>
+    <workbookView xWindow="2580" yWindow="500" windowWidth="28040" windowHeight="16940" activeTab="1" xr2:uid="{31371ACA-339D-F64C-9977-84D6DF8EF93B}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="scale" sheetId="1" r:id="rId1"/>
+    <sheet name="points-per-assignment" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="34">
   <si>
     <t>Score</t>
   </si>
@@ -105,6 +106,39 @@
   </si>
   <si>
     <t>Below 60</t>
+  </si>
+  <si>
+    <t>Assignment category</t>
+  </si>
+  <si>
+    <t>Number of assignments</t>
+  </si>
+  <si>
+    <t>Module assignments</t>
+  </si>
+  <si>
+    <t>Recitations</t>
+  </si>
+  <si>
+    <t>Class reflections</t>
+  </si>
+  <si>
+    <t>Capstone plan</t>
+  </si>
+  <si>
+    <t>Capstone assignment</t>
+  </si>
+  <si>
+    <t>Points per assignment</t>
+  </si>
+  <si>
+    <t>Total number of points</t>
+  </si>
+  <si>
+    <t>8 (you pick which ones to do)</t>
+  </si>
+  <si>
+    <t>10 (you pick which ones to do)</t>
   </si>
 </sst>
 </file>
@@ -160,9 +194,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -200,7 +234,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -306,7 +340,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -448,7 +482,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -558,4 +592,106 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A2918DB6-69F5-C446-BD6D-A14FC1703D9B}">
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="18.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.5" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B2">
+        <v>4</v>
+      </c>
+      <c r="C2">
+        <v>8</v>
+      </c>
+      <c r="D2">
+        <f>B2*C2</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4">
+        <v>2</v>
+      </c>
+      <c r="D4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5">
+        <v>1</v>
+      </c>
+      <c r="C5">
+        <v>10</v>
+      </c>
+      <c r="D5">
+        <f>B5*C5</f>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>29</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6">
+        <v>30</v>
+      </c>
+      <c r="D6">
+        <f>B6*C6</f>
+        <v>30</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>